<commit_message>
fill 300 ta 390
</commit_message>
<xml_diff>
--- a/splited_sound_with_noise/splited_sound_with_noisesplited_sound_with_noise .xlsx
+++ b/splited_sound_with_noise/splited_sound_with_noisesplited_sound_with_noise .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0project\megacom\speech\splited_sound_with_noise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA6C816-C587-4D14-84C8-B1F00198E75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E07D9F-F4C9-413A-BA28-6B6340657096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="2610" windowWidth="20085" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="990" yWindow="3180" windowWidth="14625" windowHeight="11820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1982" uniqueCount="1978">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2108" uniqueCount="2100">
   <si>
     <t>audio</t>
   </si>
@@ -5573,9 +5573,6 @@
     <t>اها چون میخواستم ببینم بشورم اینارو یا نه  میشورید پس حتما دیگه</t>
   </si>
   <si>
-    <t>دو کیلو و نیم فیله مرغ باشه  فیله مرغ وی آی پیا</t>
-  </si>
-  <si>
     <t>اشکال نداره چشم دس شما درد نکنه میام *</t>
   </si>
   <si>
@@ -5642,9 +5639,6 @@
     <t>زعفرونو اینا چنده بسته ایی چند میشه اینا</t>
   </si>
   <si>
-    <t xml:space="preserve"> بعد عع ببخشید کارت خوان هم دارید همونجا حساب کنیم</t>
-  </si>
-  <si>
     <t>ارهه من الان خودمم دوبار قبل از این باهاتون تماس گرفتم جواب ندادین</t>
   </si>
   <si>
@@ -5795,18 +5789,12 @@
     <t>همون درمونگاه ولی عصر  قبلش خب فروشگاه ماس</t>
   </si>
   <si>
-    <t xml:space="preserve">حالا باید بگیم ینی ما  الان موخام یارو برا ناهار ساعت یک من هنو دارم سرم گرمه دیدی  مغازم آبروم رفت </t>
-  </si>
-  <si>
     <t xml:space="preserve">* گوشت چرخ کرده که سفارش داده بودین </t>
   </si>
   <si>
     <t xml:space="preserve">بله جناب ملایی کیا  هستم هردو خروجی چنده </t>
   </si>
   <si>
-    <t xml:space="preserve">* فقط آقای بهرامی گفتن که </t>
-  </si>
-  <si>
     <t xml:space="preserve">یه عدد دوتا سینه است تیکه نکردی درسته اره  </t>
   </si>
   <si>
@@ -5855,9 +5843,6 @@
     <t>چش یکو دویستش خب گوساله باشه هشصد گرمش گوسفندی باشه</t>
   </si>
   <si>
-    <t>در خدمتتون آقایی هستیم سلامت باشید ممنونم مرسی قربان شما  خدانگه دار * *</t>
-  </si>
-  <si>
     <t xml:space="preserve">سلام  سلام فقط یه ساعت میتونید اعلام کنید اگه نیومدید من بعدش بفروشم </t>
   </si>
   <si>
@@ -5906,21 +5891,12 @@
     <t>اره هستش  مرغ هستش هم مرغ ساوانا داریم هم مرغ معمولی سپید گوشت</t>
   </si>
   <si>
-    <t>آقای عباسی هستم خیلی خب میام خدمتتون میام خدمتتون ممنونم عزیزم ممنونم خدافظ</t>
-  </si>
-  <si>
     <t>چون به حسنم گفتم حسن گفت زودتر بفرستین ما همینجا رد کنیم گفتم باش</t>
   </si>
   <si>
-    <t>دیگم بانک مسکن به نام آوا بتن روش نوشته جا نمونده اینجا</t>
-  </si>
-  <si>
     <t xml:space="preserve">* میرم با بچه خام پایگاه قدیم میگم بفرستن براتون </t>
   </si>
   <si>
-    <t>سلامت باشین از گوشت اطمینان تماس گرفتم خدمتتون آه *</t>
-  </si>
-  <si>
     <t>پس من دیگه نیام خودم اونجا دیگه بچه ها میارن واسم درسته</t>
   </si>
   <si>
@@ -5936,21 +5912,12 @@
     <t>کی بیام بیام عع فامیل شریفتون علیزاده</t>
   </si>
   <si>
-    <t>ممنون دستتون درد نکنه حتما سفارش بکنید به آقا سجاد حسین خانم حسین زاده زنگ زدن ممنون مرس</t>
-  </si>
-  <si>
     <t xml:space="preserve">عع چهار قسمتشو پوستش کنده بشه سر بالا زده بشه </t>
   </si>
   <si>
     <t>یدونه درشت هست حوس حول و حوش دو سه کلیویه مشکلی نداره اون</t>
   </si>
   <si>
-    <t xml:space="preserve">پس یک  سینه رو اسلایسی کنید حالت شنسلی لطف کنید بفرستید </t>
-  </si>
-  <si>
-    <t>ممنونم مرسی آقا مچکرم خواهش میکنم *</t>
-  </si>
-  <si>
     <t>البته نه هنوز هس جلال باشه اگه دستش خالی بود میدم بزنه اوکیه اره لطفن حتمن انجام بده حتما ایم فیله رو بگو زود بره من بیاد بده من دارم  من نزدیک مغازم</t>
   </si>
   <si>
@@ -5967,6 +5934,405 @@
   </si>
   <si>
     <t xml:space="preserve">مرغ معمولی اره هستش مرغ ساوانام هس فقط اگه </t>
+  </si>
+  <si>
+    <t xml:space="preserve">حالا باید بگیم ینی ما  الان موخام یارو برا ناهار ساعت یک من هنو دارم سرم گرمه دیدی  مغازم ابروم رفت </t>
+  </si>
+  <si>
+    <t xml:space="preserve">* فقط اقای بهرامی گفتن که </t>
+  </si>
+  <si>
+    <t>دو کیلو و نیم فیله مرغ باشه  فیله مرغ وی ای پیا</t>
+  </si>
+  <si>
+    <t>در خدمتتون اقایی هستیم سلامت باشید ممنونم مرسی قربان شما  خدانگه دار * *</t>
+  </si>
+  <si>
+    <t>اقای عباسی هستم خیلی خب میام خدمتتون میام خدمتتون ممنونم عزیزم ممنونم خدافظ</t>
+  </si>
+  <si>
+    <t>دیگم بانک مسکن به نام اوا بتن روش نوشته جا نمونده اینجا</t>
+  </si>
+  <si>
+    <t>سلامت باشین از گوشت اطمینان تماس گرفتم خدمتتون اه *</t>
+  </si>
+  <si>
+    <t>ممنون دستتون درد نکنه حتما سفارش بکنید به اقا سجاد حسین خانم حسین زاده زنگ زدن ممنون مرس</t>
+  </si>
+  <si>
+    <t>ممنونم مرسی اقا مچکرم خواهش میکنم *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اره یه مشتریم به اسم اقای رستم داریم یک عع شماره تماسم لطف میکنید نهصدو بیست و یک </t>
+  </si>
+  <si>
+    <t>دهقان هستم میخاستم بگم که من دز</t>
+  </si>
+  <si>
+    <t>خب بیام وایستم که شب بهم میدین من با گوشت دیگه باید قاتی کنم که به فردا صب نکشه میام همون دور و بره</t>
+  </si>
+  <si>
+    <t>بعد عزیز من ببخشین شما چون زنگ زدی دوتا ماهیچه سر دستم من میخام میتونی اضافه کنی برام</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عع من براتون سفارش رو اوردم بعد یسری دستور مونده بود الان خاستم ببینم </t>
+  </si>
+  <si>
+    <t>من قبلا با اقای حیدریان چیز میکردم ایشون میاورد دم خونه برام همرو</t>
+  </si>
+  <si>
+    <t>**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قربان شما به نام اقای روشن فرمودین ناظم ناظم مدرسه </t>
+  </si>
+  <si>
+    <t>عع چارشنبه پنجشنبه کله پاچه میخاین</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* گفتن که شما زنگ بزنین برات میفرستین من میرم حساب میکنم </t>
+  </si>
+  <si>
+    <t>خب توراه فردا میتونم بیارم اشکال نداره نداره بیاید حاج اقا اشکال نداره باشه تشریف بیارید</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> بعد عع ببخشید کارت خان هم دارید همونجا حساب کنیم</t>
+  </si>
+  <si>
+    <t>نه فرقی نمیکنه اگه نگا اگه رویه بوی ماهی حساسین که مثلا ماهی سی بس داریم میتونین اونو ببرین کلا ماهیش بدون بوه ولی اگه زیا مثلا اون بوش مشکلی نداره ماهی زیاد دارم  هم ماهی شوریده هس خیلی ماهیه با کیفیتیه خیلی خوش طمیه بد</t>
+  </si>
+  <si>
+    <t>اقای قاسم زاده بله سفارشتون حاظره جناب باش میام خدمتتون مرسی لطف دارین خدافظ خدا</t>
+  </si>
+  <si>
+    <t>خب حاج خانوم نگا کنید دست ما نیس خب  ما به کارگاه میگیم میگیم کوچیک ترین شقه رو برا شما بزارن خب</t>
+  </si>
+  <si>
+    <t>ببخشین میخاستم زنگ بزنم فراموش کردم شرمنده ببخشید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">با کیفیت تر و بهتر حالا نمیدونم تاحالا تست کردین کدومش فیله دار  </t>
+  </si>
+  <si>
+    <t>عم دستگاه روشنه داخل مغازه اره ببخشین عذرخاهم صداتون بد میومد شفیعی دوباره ش شفیعی اقا</t>
+  </si>
+  <si>
+    <t>پس فردا میام میگیرم دست شما فقط زود یک برام میفرستین یک هفده</t>
+  </si>
+  <si>
+    <t>نیاورانه الان حضور ذهن ندارم نقشه نیاوران چند میشه نگا طلاییه شرق *</t>
+  </si>
+  <si>
+    <t>نه بدون استخون خورشتی بشه استخونش جدا</t>
+  </si>
+  <si>
+    <t xml:space="preserve">میگم باید سفارش بدم براتون اره اوکیش میکنم براتون </t>
+  </si>
+  <si>
+    <t xml:space="preserve">حالا اگه شد شونزه تشریف بیارین وگرنه که باز بدظهر میام * </t>
+  </si>
+  <si>
+    <t>* اماده کنید دره چیز</t>
+  </si>
+  <si>
+    <t>اره اره کلا شیش قسمت بشه باشه</t>
+  </si>
+  <si>
+    <t>بلدرچین روزای فرد میاد دیروز اورده بودیم تموم شد باز ایشالا فردا میاد</t>
+  </si>
+  <si>
+    <t>نعیمیم عزیزم خوبی جانم اقای نعیمی بفرمایین درخدممتونم قربونت برم یه زحمت میکشید به بچه ها بگید میتونن اون سی تا رون چارصد گرمی رو به من برسونن</t>
+  </si>
+  <si>
+    <t>با پونصد گرمم قلوه گاه پس چرخ کرده لطف کنید</t>
+  </si>
+  <si>
+    <t>سلام جناب عابدی شبتون بخیر خوبین در سلامت باشین ممنونم سلامت باشی از گوشت اطمینان تماس گرفتمم خدمتتون</t>
+  </si>
+  <si>
+    <t>خب بگین من الان میام خودم حضوری وردار میام تا یک ده دقیقه یه رب دیگه میام خدمتتون</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اره مرغم هستش فقط مرغا یک مقداری سایز متوسطاش تموم شده یا ریزه یا یه مقدار درشت ازین </t>
+  </si>
+  <si>
+    <t>حالا خو سعی کن یکم کوچیک ترشو برام اگر میشه دوتا نگه داری</t>
+  </si>
+  <si>
+    <t>الان بزار من بنویسم حاج اقا براتون *</t>
+  </si>
+  <si>
+    <t>ما که خانم قصابیه ولی میوه فروشیم هسته معرفی کنیم بله ایجا هستا</t>
+  </si>
+  <si>
+    <t>ولی اگر که میبینید چیزه فردارم مشکلی نیستش رسید برام</t>
+  </si>
+  <si>
+    <t>دستت درد نکنه باز میام اونجا بهت سفارششو ک دادم همونجا میگیرم</t>
+  </si>
+  <si>
+    <t>میگم چقده اینو اپدیت عم قیمتاش اشتبایه یا ماهی جنوبا</t>
+  </si>
+  <si>
+    <t>بعد واستون بوقلمون چرخ کرده میزاشتینم یک دونه میزاشتین یا  سس نیزاشتین یادم نیستش</t>
+  </si>
+  <si>
+    <t>اره خب بریم اول سفارش اول یک رون با چربی میخاد خورشتی ریز شه</t>
+  </si>
+  <si>
+    <t>خب چ حالا هس دنبه هس ببرم جان اره اره منظور هستش یک دنبه کامل سفارش بدی اونجا نزدیک ده کیلو هستش</t>
+  </si>
+  <si>
+    <t>* چقد میخاین خانم سعیدی</t>
+  </si>
+  <si>
+    <t>خب اگه همون قیمته اره پوستشو بکنه دستش درد نکنه *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ساعت یک تا سه م خوبه احتمالا قب اره لش خودم میام پس میگیرم دیگه </t>
+  </si>
+  <si>
+    <t>بابت سفارش که داده بودید سه *</t>
+  </si>
+  <si>
+    <t>اها چون وقتی که موخام بیام باز مادرم موخام بیارم اون سری اومدم گفتن تموم کرده باز نمیتونه</t>
+  </si>
+  <si>
+    <t>بعد عع برا برا چه تایمی میخاین *</t>
+  </si>
+  <si>
+    <t>میخاین اگه مرغ تازه ترمیاد چرا مرغ امروز مرغه سمت ساعت یازده ده یازده صب میاد</t>
+  </si>
+  <si>
+    <t>و اینکه ععم دوکیلو نیم گوساله</t>
+  </si>
+  <si>
+    <t>* صالحیم میخاستم ببینم که رونو جانم سینه بوقلمون دارین</t>
+  </si>
+  <si>
+    <t>شینسل مرغش که انگار میشه  همون جوجه کبابش دویستو سی و هف تومنه</t>
+  </si>
+  <si>
+    <t>دو عدد شینسل چیکار بشه اینا سالم باشه یا اینام میخاین تیکه ای چیزی بشه نه اینا سالم باشه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">پس یک  سینه رو اسلایسی کنید حالت شنیسلی لطف کنید بفرستید </t>
+  </si>
+  <si>
+    <t>بله بله ماهیایی که اوردیم همه مال جنوبه *</t>
+  </si>
+  <si>
+    <t>اها دسته درسته دقیق چون چون پیروز شما گفتید دیروز دیروز گفتین ک</t>
+  </si>
+  <si>
+    <t>بله هشصدو هفتادو هشت</t>
+  </si>
+  <si>
+    <t>* با هم دیگه چیز کنید جد جدا کنید چیز چرخ کنین من میام میبرم</t>
+  </si>
+  <si>
+    <t>هش میکنم ببخشید تماس گرفتید برای اینکه ماهی گف قرار بود تیکه کنن امادس بیام ببرم میخاستم ببینم من میتونید برام بفرستین عع</t>
+  </si>
+  <si>
+    <t>* جسارتن اومدید خودتون معرفی کنید که شما اقای عباسی این دیگه اره</t>
+  </si>
+  <si>
+    <t>دست میخاستم اینا در حد مثلا دو کیلو دو کیلو و خورده ای</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الان برا دوک امروز براشون مرغ نیومده میخان وایسید </t>
+  </si>
+  <si>
+    <t>ساوانا صدو بیستو هفتو نهصده مرغ معمولی هشتادو پنجو هفصده</t>
+  </si>
+  <si>
+    <t>میز بشه پس شما یکاری کنید شما همین شماره ای که گرفتینو داخلی پنجو بگیرین به خوده اقای میرشکار وصل میشه اها با</t>
+  </si>
+  <si>
+    <t>الو سلام بزرگوار وقتت *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اون ها اون ها اره حاظره فقط چیزش حاظر نیس دیگه فیلشو خیلی شلوغ بود مغازه من به بچه هام گفتم </t>
+  </si>
+  <si>
+    <t>بعد الان منم مرغ گرفتم بعد دفه سومه همیشم میگم هس نکنن برا من بعد تا میام خونه بسته بندی کنم میبینم همرو پوست کردن به من برا سرخ کردن میخاس</t>
+  </si>
+  <si>
+    <t>سه عدد باشه خورشتی خودمونم هستا اگه میخاین حالا خب</t>
+  </si>
+  <si>
+    <t>فردا نه تا دو نه تا دو</t>
+  </si>
+  <si>
+    <t>مگه اینکه حضوری بیان اینجا بچه ها کارتون رو راه بندازن چون یه مقداری سفارشا زیاده</t>
+  </si>
+  <si>
+    <t>این هشتادو نهه معمولی اون صدو بیستو هفته ولی خب از لحاظ طعمیو کیفیت بهترین مرغه کشوره</t>
+  </si>
+  <si>
+    <t xml:space="preserve">باش پس بگو بزنن من واریز میکنم اس ام اس میکنم خدمتتون </t>
+  </si>
+  <si>
+    <t>بفرمایید که عع م عع قیمتش راستی قیمتا چند بوده ک من صب نگا نکردم *</t>
+  </si>
+  <si>
+    <t>قزلا قزلای مال رودخونه ایه مال سمت درگزه</t>
+  </si>
+  <si>
+    <t>* الان حاظر بکنید دوازده تا یک بیام بگیرم نمیشه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عع شیره بعد دیگه </t>
+  </si>
+  <si>
+    <t>پس خب چند میشه قیمتشو میخام بگم به این بنده خدایی که میخاد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قلم گوساله موجود نداریم ولی میتونید شما سفارش بدین ما هر وقت </t>
+  </si>
+  <si>
+    <t>بعد گوشت گوسفندی قلوه گاهو گوسفندی دارین که رونو اینا اره قلوه گاه گوسفندیم هستش</t>
+  </si>
+  <si>
+    <t>حاج اقا شما فاکتوره کلشو صندوق حساب کردین دادیم خدمتون دیگه **</t>
+  </si>
+  <si>
+    <t>خب فدا سرت من دیروز دیروز با اقا صحبت کردم گفت شاید شاید این این شعبتون چیه اسمه وکیل اباده هی اسمشو یادم میره طلایی *</t>
+  </si>
+  <si>
+    <t>* خب الانه بیام خدمتتون *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">گفتین اگر ماهی قزل نیومده برام خانم قطبی </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ساوانا حداکثر بزرگترینش دیگه دو کیلوه همه مرغای ساوانا نه نه یکو هشصد * </t>
+  </si>
+  <si>
+    <t>سلام خانم اقا یک مرغی از شما گرفتیم دوتا فاکتور دادین</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مرسی یه شیش تا سینه مرغ هم این مثل همیشه میخام دیگه تا قرار بود متوجه خودتون نظارت کنید دیگه درسته  </t>
+  </si>
+  <si>
+    <t>اره چون همیشه زرد رنگ *</t>
+  </si>
+  <si>
+    <t>بین یازده تا سیزده کیلو اخ کوچیک ترشو ندارین کوچیک ترشو</t>
+  </si>
+  <si>
+    <t>یدونه درست هست حوس حول و حوش دو سه کلیویه مشکلی نداره اون</t>
+  </si>
+  <si>
+    <t>گله ایه نه خب من میخام سر کار برم من تا یک بیشتر  حاج اقا ستم خونه *</t>
+  </si>
+  <si>
+    <t xml:space="preserve">باشه پس عذرخاهم باز خدمتتون تماس میگیرم مرسی  </t>
+  </si>
+  <si>
+    <t>برای همون دو کیلو کافی باشه خیلی نمیخام مرغش زیاد باشه</t>
+  </si>
+  <si>
+    <t>یازده دوازده بسیار خب عمر دیگه باشه</t>
+  </si>
+  <si>
+    <t>خب شما بعد خبر میدین که یعنی ما کی بیایم چجوره *</t>
+  </si>
+  <si>
+    <t>خب بنویسن سفید دی میایم تا من ناهار هنو نخوردم ناهار بخورم می</t>
+  </si>
+  <si>
+    <t>باش باش این یارو خیلی شاکی شده واسه همین دمت گرم مرسی عزیزم خدافظ</t>
+  </si>
+  <si>
+    <t>ا الان صدا خوب شد میگم خیلی خب از  اطمینان خدمتتون تماس گرفتم سفارش مغز گوساله که گفته بودین رسیده گفتم میتونین بیاین ببرین</t>
+  </si>
+  <si>
+    <t>عع یک سفارش برا فردا میخاستم انجام بدین برام پس یک تیکده خوبی متاسفانه هی کنسلی خورده میونش این کار انجام بدیم</t>
+  </si>
+  <si>
+    <t>بین وکیل اباده شصتو یکو شصتو سه و شصتو یک یا شصت سه</t>
+  </si>
+  <si>
+    <t>من عع وکیلی هستم مزاحمتون میشم عع صبح اومدن خدمتتون برقا قط شد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* اینا میام میگیرم سه تا </t>
+  </si>
+  <si>
+    <t xml:space="preserve">عع بفرمایید عع کله پاچه چارشنبه یا شنبه هم دارین یا نه </t>
+  </si>
+  <si>
+    <t>یه لحظه اقا سجاد سینه مرغی حدود بله بله</t>
+  </si>
+  <si>
+    <t>شیر باز انشالا باید ببینیم بار بعدیش کی میاد چون هفته یبار بیشتر نمیاد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">یک دو سه ساعت دیگه خبر بگیرین بهتون بگم </t>
+  </si>
+  <si>
+    <t>اقایه افشانه عع</t>
+  </si>
+  <si>
+    <t>فقط جسارتا پیک عمده بین  ساعت یک ظهر تا چار بعده ظهره کلا</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*سلامت باشین اقا من اسلامی هستم دیروز عصر اومدم یک سفارش گذاشتم قرار شد پیک واسم بیاره میخاستم ببینم امروز میاره پیک یا نه سفارشمو </t>
+  </si>
+  <si>
+    <t>این عع پیکامون بین ساعت دو تا چاره بین اون ساعت براتون میاره</t>
+  </si>
+  <si>
+    <t>الان صداتون قط و وصل میشه می چرا ضعیف تر عع میگم *</t>
+  </si>
+  <si>
+    <t>اره اره پنج خوبه فقط درشتیش برام خیلی مهمه ها لطفا خیلی درشت با</t>
+  </si>
+  <si>
+    <t>هر دو بسته رو دیگه اره هر دو بسته رو چیزی توش نزنین فقط</t>
+  </si>
+  <si>
+    <t xml:space="preserve">بهزاد هستم اگه محبت کنید برا من یک کیلو قیمه ای </t>
+  </si>
+  <si>
+    <t>مرغ بدون هرمون میخاستم مرغ ساوانا</t>
+  </si>
+  <si>
+    <t xml:space="preserve">پونصد تومنه پونصدو حالا شصت پونصدو چل پونصدو نود </t>
+  </si>
+  <si>
+    <t>خو الان برقا رفته خب مشکلی ندارین الان یا برقا اومده جایه شما الان</t>
+  </si>
+  <si>
+    <t>فدات بشم دستتم درد نکنه ممنونم بکل خدافظ قربانت خدافظ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">خب میگم خانم مشتری حضوری بیاین که اونا رو بزارن کنار سفارش شما رو بدهن خیلی </t>
+  </si>
+  <si>
+    <t>باشه چشم چشم فقط کی تشریف میارید جناب قرایی شما</t>
+  </si>
+  <si>
+    <t>عع سه عدد مرغه یکو دویست و دویستی خب</t>
+  </si>
+  <si>
+    <t>سرافرازان تویه گوگل سرچ کنید ادرسشو براتون میاره</t>
+  </si>
+  <si>
+    <t>حتما این پاچه گوسفندی اومده اگه میخای تشیف بیارین ببرین</t>
+  </si>
+  <si>
+    <t>ببخشید شما * یه رب به یازده سفارش گوشت دادم حضوری یعنی همسرم اومد خب الان رفتم تو لینک چه شکلیه سایت</t>
+  </si>
+  <si>
+    <t>تمام پوستشو کند یعنی یه تیکه پوست معمولی ریزم ندارن که توش انقد</t>
+  </si>
+  <si>
+    <t>از مجموعه گوشت اطمینان مزاحمتون میشم شعبه طلاییه دو</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سلام و خسته نباشید </t>
   </si>
 </sst>
 </file>
@@ -6411,7 +6777,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6423,7 +6789,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1857</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -6435,7 +6801,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -6447,7 +6813,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1859</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -6459,7 +6825,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1860</v>
+        <v>1859</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -6471,7 +6837,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1861</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -6483,7 +6849,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -6495,7 +6861,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>1863</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -6507,7 +6873,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>1864</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -6519,7 +6885,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1865</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -6531,7 +6897,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>1866</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -6543,7 +6909,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>1867</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -6564,7 +6930,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>1868</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -6576,7 +6942,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>1869</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -6588,7 +6954,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>1870</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -6600,7 +6966,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>1871</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -6612,7 +6978,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>1872</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -6624,7 +6990,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>1873</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -6636,7 +7002,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>1874</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -6648,7 +7014,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>1875</v>
+        <v>1873</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -6660,7 +7026,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>1917</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -6672,7 +7038,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>1918</v>
+        <v>1916</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -6684,7 +7050,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>1876</v>
+        <v>1874</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -6696,7 +7062,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>1877</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -6708,7 +7074,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>1878</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -6720,7 +7086,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>1879</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -6732,7 +7098,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>1880</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -6744,7 +7110,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>1881</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -6756,7 +7122,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>1919</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -6768,7 +7134,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>1882</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -6780,7 +7146,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>1896</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -6792,7 +7158,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>1883</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -6804,7 +7170,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>1884</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -6816,7 +7182,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>1894</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -6828,7 +7194,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>1895</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -6840,7 +7206,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>1885</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -6852,7 +7218,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>1886</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -6864,7 +7230,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>1887</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -6876,7 +7242,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>1888</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -6888,7 +7254,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>1920</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -6900,7 +7266,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>1921</v>
+        <v>1918</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -6912,7 +7278,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>1889</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -6924,7 +7290,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>1890</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -6936,7 +7302,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>1922</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -6948,7 +7314,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>1891</v>
+        <v>1889</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -6960,7 +7326,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>1892</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -6972,7 +7338,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>1923</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -6984,7 +7350,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>1893</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -6996,7 +7362,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>1924</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -7008,7 +7374,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -7020,7 +7386,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>1925</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -7032,7 +7398,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>1897</v>
+        <v>1895</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -7044,7 +7410,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>1898</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -7056,7 +7422,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>1899</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -7068,7 +7434,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>1900</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -7080,7 +7446,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>1901</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -7092,7 +7458,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>1902</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -7104,7 +7470,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>1903</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -7116,7 +7482,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>1926</v>
+        <v>1922</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -7128,7 +7494,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>1904</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -7140,7 +7506,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>1905</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -7152,7 +7518,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>1906</v>
+        <v>1904</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -7164,7 +7530,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>1907</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -7176,7 +7542,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>1908</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -7188,7 +7554,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>1927</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -7200,7 +7566,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>1909</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -7212,7 +7578,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>1910</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -7224,7 +7590,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>1911</v>
+        <v>1909</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -7236,7 +7602,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>1912</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -7248,7 +7614,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>1913</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -7260,7 +7626,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>1914</v>
+        <v>1912</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -7272,7 +7638,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -7284,7 +7650,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>1915</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -7296,7 +7662,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>1956</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -7308,7 +7674,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>1928</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -7320,7 +7686,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>1916</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -8433,7 +8799,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>1846</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
@@ -8445,7 +8811,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>1847</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -8457,7 +8823,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>1848</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
@@ -8469,7 +8835,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
@@ -8481,7 +8847,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -8493,7 +8859,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -8505,7 +8871,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
@@ -8517,7 +8883,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C208" s="1" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
@@ -8529,7 +8895,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
@@ -8541,10 +8907,10 @@
         <v>Play Audio</v>
       </c>
       <c r="C210" s="1" t="s">
-        <v>1929</v>
+        <v>1925</v>
       </c>
       <c r="F210" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
@@ -8556,7 +8922,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C211" s="1" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
@@ -8568,7 +8934,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C212" s="1" t="s">
-        <v>1930</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
@@ -8580,7 +8946,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C213" s="1" t="s">
-        <v>1931</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
@@ -8592,7 +8958,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C214" s="1" t="s">
-        <v>1932</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
@@ -8604,7 +8970,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>1933</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.25">
@@ -8616,7 +8982,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C216" s="1" t="s">
-        <v>1934</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
@@ -8628,7 +8994,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C217" s="1" t="s">
-        <v>1935</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
@@ -8640,7 +9006,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C218" s="1" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
@@ -8652,7 +9018,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C219" s="1" t="s">
-        <v>1936</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.25">
@@ -8664,7 +9030,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C220" s="1" t="s">
-        <v>1937</v>
+        <v>1933</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
@@ -8676,7 +9042,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C221" s="1" t="s">
-        <v>1938</v>
+        <v>1934</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
@@ -8688,7 +9054,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C222" s="1" t="s">
-        <v>1939</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
@@ -8700,7 +9066,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C223" s="1" t="s">
-        <v>1940</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
@@ -8712,7 +9078,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>1941</v>
+        <v>1936</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
@@ -8724,7 +9090,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C225" s="1" t="s">
-        <v>1942</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
@@ -8736,7 +9102,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C226" s="1" t="s">
-        <v>1943</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
@@ -8748,7 +9114,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C227" s="1" t="s">
-        <v>1944</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
@@ -8760,7 +9126,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C228" s="1" t="s">
-        <v>1945</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
@@ -8772,7 +9138,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C229" s="1" t="s">
-        <v>1946</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
@@ -8784,7 +9150,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C230" s="1" t="s">
-        <v>1947</v>
+        <v>1942</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
@@ -8796,7 +9162,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C231" s="1" t="s">
-        <v>1948</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
@@ -8808,7 +9174,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>1949</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
@@ -8820,7 +9186,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>1950</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -8832,7 +9198,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>1951</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
@@ -8844,7 +9210,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>1952</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
@@ -8856,7 +9222,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>1953</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
@@ -8868,7 +9234,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C237" s="1" t="s">
-        <v>1954</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
@@ -8880,7 +9246,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C238" s="1" t="s">
-        <v>1955</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
@@ -8892,7 +9258,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>1957</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
@@ -8904,7 +9270,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C240" s="1" t="s">
-        <v>1958</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
@@ -8916,7 +9282,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C241" s="1" t="s">
-        <v>1959</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
@@ -8928,7 +9294,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C242" s="1" t="s">
-        <v>1960</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
@@ -8940,7 +9306,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>1961</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
@@ -8952,7 +9318,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C244" s="1" t="s">
-        <v>1962</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
@@ -8964,7 +9330,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>1963</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
@@ -8976,7 +9342,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>1964</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
@@ -8988,7 +9354,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C247" s="1" t="s">
-        <v>1965</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
@@ -9000,7 +9366,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C248" s="1" t="s">
-        <v>1966</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
@@ -9012,7 +9378,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C249" s="1" t="s">
-        <v>1967</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
@@ -9024,7 +9390,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C250" s="1" t="s">
-        <v>1968</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
@@ -9036,7 +9402,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C251" s="1" t="s">
-        <v>1969</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
@@ -9048,7 +9414,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C252" s="1" t="s">
-        <v>1970</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
@@ -9060,7 +9426,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>1971</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
@@ -9072,7 +9438,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C254" s="1" t="s">
-        <v>1972</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
@@ -9084,7 +9450,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C255" s="1" t="s">
-        <v>1973</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
@@ -9096,7 +9462,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C256" s="1" t="s">
-        <v>1974</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
@@ -9108,7 +9474,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>1975</v>
+        <v>1964</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
@@ -9120,7 +9486,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>1976</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
@@ -9132,7 +9498,7 @@
         <v>Play Audio</v>
       </c>
       <c r="C259" s="1" t="s">
-        <v>1977</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
@@ -9143,6 +9509,9 @@
         <f>HYPERLINK("1739961707_8_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C260" s="1" t="s">
+        <v>1976</v>
+      </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" s="4" t="s">
@@ -9152,6 +9521,9 @@
         <f>HYPERLINK("1739962376_0_SPK_1_20250215_v2.1739611648.2264164.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C261" s="1" t="s">
+        <v>1977</v>
+      </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="4" t="s">
@@ -9161,6 +9533,9 @@
         <f>HYPERLINK("1739962476_12_SPK_1_20250213_v2.1739457460.2227454.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C262" s="1" t="s">
+        <v>1978</v>
+      </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" s="4" t="s">
@@ -9170,6 +9545,9 @@
         <f>HYPERLINK("1739962974_5_SPK_1_20250215_v2.1739611272.2263888.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C263" s="1" t="s">
+        <v>1854</v>
+      </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" s="4" t="s">
@@ -9179,6 +9557,9 @@
         <f>HYPERLINK("1739962440_4_SPK_1_20250213_v2.1739467465.2237596.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C264" s="1" t="s">
+        <v>1979</v>
+      </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" s="4" t="s">
@@ -9188,6 +9569,9 @@
         <f>HYPERLINK("1739962841_1_SPK_1_20250213_v2.1739462017.2231984.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C265" s="1" t="s">
+        <v>1854</v>
+      </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" s="4" t="s">
@@ -9197,6 +9581,9 @@
         <f>HYPERLINK("1739962231_0_SPK_1_20250216_v2.1739706913.2331299.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C266" s="1" t="s">
+        <v>1980</v>
+      </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" s="4" t="s">
@@ -9206,6 +9593,9 @@
         <f>HYPERLINK("1739961678_14_SPK_1_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C267" s="1" t="s">
+        <v>1854</v>
+      </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" s="4" t="s">
@@ -9215,6 +9605,9 @@
         <f>HYPERLINK("1739962861_31_SPK_1_20250216_v2.1739695895.2308017.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C268" s="1" t="s">
+        <v>1981</v>
+      </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" s="4" t="s">
@@ -9224,6 +9617,9 @@
         <f>HYPERLINK("1739962896_3_SPK_1_20250216_v2.1739707901.2331813.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C269" s="1" t="s">
+        <v>1982</v>
+      </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" s="4" t="s">
@@ -9233,6 +9629,9 @@
         <f>HYPERLINK("1739961707_7_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C270" s="1" t="s">
+        <v>1983</v>
+      </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" s="4" t="s">
@@ -9242,6 +9641,9 @@
         <f>HYPERLINK("1739962709_1_SPK_1_20250217_v2.1739780534.2356086.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
+      <c r="C271" s="1" t="s">
+        <v>1984</v>
+      </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" s="4" t="s">
@@ -9251,8 +9653,11 @@
         <f>HYPERLINK("1739962503_17_SPK_1_20250215_v2.1739623381.2279172.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C272" s="1" t="s">
+        <v>1985</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" s="4" t="s">
         <v>274</v>
       </c>
@@ -9260,8 +9665,11 @@
         <f>HYPERLINK("1739962906_12_SPK_1_20250216_v2.1739710661.2333661.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C273" s="1" t="s">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" s="4" t="s">
         <v>275</v>
       </c>
@@ -9269,8 +9677,11 @@
         <f>HYPERLINK("1739962753_11_SPK_1_20250217_v2.1739783930.2360950.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C274" s="1" t="s">
+        <v>1988</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" s="4" t="s">
         <v>276</v>
       </c>
@@ -9278,8 +9689,11 @@
         <f>HYPERLINK("1739962897_2_SPK_1_20250217_v2.1739810129.2391951.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C275" s="1" t="s">
+        <v>1989</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" s="4" t="s">
         <v>277</v>
       </c>
@@ -9287,17 +9701,23 @@
         <f>HYPERLINK("1739962597_12_SPK_1_20250215_v2.1739624662.2279909.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C276" s="1" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="B277" s="6" t="str">
+      <c r="B277" s="7" t="str">
         <f>HYPERLINK("1739962390_2_SPK_0_20250213_v2.1739460813.2230789.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C277" s="1" t="s">
+        <v>1991</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
         <v>279</v>
       </c>
@@ -9305,17 +9725,23 @@
         <f>HYPERLINK("1739962753_9_SPK_1_20250217_v2.1739783930.2360950.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C278" s="1" t="s">
+        <v>1992</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="B279" s="6" t="str">
+      <c r="B279" s="7" t="str">
         <f>HYPERLINK("1739962930_5_SPK_0_20250215_v2.1739635851.2285514.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C279" s="1" t="s">
+        <v>1993</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" s="4" t="s">
         <v>281</v>
       </c>
@@ -9323,8 +9749,11 @@
         <f>HYPERLINK("1739962763_4_SPK_1_20250215_v2.1739634735.2284891.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C280" s="1" t="s">
+        <v>1994</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" s="4" t="s">
         <v>282</v>
       </c>
@@ -9332,8 +9761,11 @@
         <f>HYPERLINK("1739962161_19_SPK_0_20250215_v2.1739603840.2258967.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C281" s="1" t="s">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" s="4" t="s">
         <v>283</v>
       </c>
@@ -9341,8 +9773,11 @@
         <f>HYPERLINK("1739962483_4_SPK_0_20250215_v2.1739598239.2256261.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C282" s="1" t="s">
+        <v>1996</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" s="4" t="s">
         <v>284</v>
       </c>
@@ -9350,8 +9785,11 @@
         <f>HYPERLINK("1739962986_3_SPK_1_20250217_v2.1739811359.2393115.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C283" s="1" t="s">
+        <v>1997</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" s="4" t="s">
         <v>285</v>
       </c>
@@ -9359,8 +9797,11 @@
         <f>HYPERLINK("1739961668_6_SPK_1_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C284" s="1" t="s">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" s="4" t="s">
         <v>286</v>
       </c>
@@ -9368,8 +9809,11 @@
         <f>HYPERLINK("1739962636_1_SPK_0_20250215_v2.1739620682.2277220.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C285" s="1" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" s="4" t="s">
         <v>287</v>
       </c>
@@ -9377,8 +9821,11 @@
         <f>HYPERLINK("1739962426_13_SPK_1_20250213_v2.1739453516.2221986.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C286" s="1" t="s">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" s="4" t="s">
         <v>288</v>
       </c>
@@ -9386,8 +9833,11 @@
         <f>HYPERLINK("1739962295_0_SPK_0_20250217_v2.1739784322.2361744.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C287" s="1" t="s">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" s="4" t="s">
         <v>289</v>
       </c>
@@ -9395,8 +9845,11 @@
         <f>HYPERLINK("1739962739_1_SPK_1_20250217_v2.1739793056.2372970.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C288" s="1" t="s">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" s="4" t="s">
         <v>290</v>
       </c>
@@ -9404,8 +9857,11 @@
         <f>HYPERLINK("1739961655_7_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C289" s="1" t="s">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" s="4" t="s">
         <v>291</v>
       </c>
@@ -9413,17 +9869,23 @@
         <f>HYPERLINK("1739962436_0_SPK_1_20250213_v2.1739461909.2231873.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C290" s="1" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="B291" s="6" t="str">
+      <c r="B291" s="7" t="str">
         <f>HYPERLINK("1739962239_9_SPK_0_20250216_v2.1739698265.2310367.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C291" s="1" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" s="4" t="s">
         <v>293</v>
       </c>
@@ -9432,7 +9894,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293" s="4" t="s">
         <v>294</v>
       </c>
@@ -9440,8 +9902,11 @@
         <f>HYPERLINK("1739962518_7_SPK_1_20250217_v2.1739793977.2374162.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C293" s="1" t="s">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294" s="4" t="s">
         <v>295</v>
       </c>
@@ -9449,17 +9914,23 @@
         <f>HYPERLINK("1739962175_4_SPK_0_20250215_v2.1739614093.2265728.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C294" s="1" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="B295" s="6" t="str">
-        <f>HYPERLINK("1739962966_3_SPK_1_20250215_v2.1739600150.2256688.wav", "Play Audio")</f>
-        <v>Play Audio</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B295" s="7" t="str">
+        <f>HYPERLINK("1739962966_3_SPK_1_20250215_v2.1739600150.2256688.C296wav", "Play Audio")</f>
+        <v>Play Audio</v>
+      </c>
+      <c r="C295" s="1" t="s">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296" s="4" t="s">
         <v>297</v>
       </c>
@@ -9467,8 +9938,11 @@
         <f>HYPERLINK("1739962598_20_SPK_1_20250215_v2.1739624662.2279909.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C296" s="1" t="s">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297" s="4" t="s">
         <v>298</v>
       </c>
@@ -9476,17 +9950,23 @@
         <f>HYPERLINK("1739962832_5_SPK_0_20250216_v2.1739711771.2334478.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C297" s="1" t="s">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="B298" s="6" t="str">
+      <c r="B298" s="7" t="str">
         <f>HYPERLINK("1739961628_4_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C298" s="1" t="s">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299" s="4" t="s">
         <v>300</v>
       </c>
@@ -9494,17 +9974,23 @@
         <f>HYPERLINK("1739962419_3_SPK_1_20250215_v2.1739617417.2275380.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C299" s="1" t="s">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="B300" s="6" t="str">
+      <c r="B300" s="7" t="str">
         <f>HYPERLINK("1739962654_9_SPK_0_20250215_v2.1739599940.2256629.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C300" s="1" t="s">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301" s="4" t="s">
         <v>302</v>
       </c>
@@ -9512,8 +9998,11 @@
         <f>HYPERLINK("1739962998_6_SPK_0_20250216_v2.1739697766.2309766.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C301" s="1" t="s">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302" s="4" t="s">
         <v>303</v>
       </c>
@@ -9521,8 +10010,11 @@
         <f>HYPERLINK("1739962494_4_SPK_1_20250217_v2.1739780189.2355491.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C302" s="1" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303" s="4" t="s">
         <v>304</v>
       </c>
@@ -9530,8 +10022,11 @@
         <f>HYPERLINK("1739962399_6_SPK_0_20250213_v2.1739454160.2223094.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C303" s="1" t="s">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304" s="4" t="s">
         <v>305</v>
       </c>
@@ -9540,7 +10035,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" s="4" t="s">
         <v>306</v>
       </c>
@@ -9548,8 +10043,11 @@
         <f>HYPERLINK("1739961624_7_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C305" s="1" t="s">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306" s="4" t="s">
         <v>307</v>
       </c>
@@ -9557,8 +10055,11 @@
         <f>HYPERLINK("1739962654_2_SPK_0_20250215_v2.1739599940.2256629.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C306" s="1" t="s">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" s="4" t="s">
         <v>308</v>
       </c>
@@ -9566,8 +10067,11 @@
         <f>HYPERLINK("1739962211_1_SPK_1_20250216_v2.1739685520.2296728.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C307" s="1" t="s">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" s="4" t="s">
         <v>309</v>
       </c>
@@ -9575,8 +10079,11 @@
         <f>HYPERLINK("1739961658_4_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C308" s="1" t="s">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A309" s="4" t="s">
         <v>310</v>
       </c>
@@ -9584,8 +10091,11 @@
         <f>HYPERLINK("1739961678_8_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C309" s="1" t="s">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" s="4" t="s">
         <v>311</v>
       </c>
@@ -9593,8 +10103,11 @@
         <f>HYPERLINK("1739962998_17_SPK_0_20250216_v2.1739697766.2309766.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C310" s="1" t="s">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" s="4" t="s">
         <v>312</v>
       </c>
@@ -9603,7 +10116,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" s="4" t="s">
         <v>313</v>
       </c>
@@ -9611,8 +10124,11 @@
         <f>HYPERLINK("1739961655_6_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C312" s="1" t="s">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" s="4" t="s">
         <v>314</v>
       </c>
@@ -9620,8 +10136,11 @@
         <f>HYPERLINK("1739962948_9_SPK_1_20250217_v2.1739802175.2383421.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C313" s="1" t="s">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" s="4" t="s">
         <v>315</v>
       </c>
@@ -9629,8 +10148,11 @@
         <f>HYPERLINK("1739961641_2_SPK_1_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C314" s="1" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" s="4" t="s">
         <v>316</v>
       </c>
@@ -9638,17 +10160,23 @@
         <f>HYPERLINK("1739962165_2_SPK_1_20250216_v2.1739692142.2303842.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C315" s="1" t="s">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="B316" s="6" t="str">
-        <f>HYPERLINK("1739962818_6_SPK_0_20250215_v2.1739613797.2265592.wav", "Play Audio")</f>
-        <v>Play Audio</v>
-      </c>
-    </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B316" s="7" t="str">
+        <f>HYPERLINK("1739962818_6_SPK_0_20250215_v2.1739613797.C3142265592.wav", "Play Audio")</f>
+        <v>Play Audio</v>
+      </c>
+      <c r="C316" s="1" t="s">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" s="4" t="s">
         <v>318</v>
       </c>
@@ -9656,8 +10184,11 @@
         <f>HYPERLINK("1739962861_6_SPK_1_20250216_v2.1739695895.2308017.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C317" s="1" t="s">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" s="4" t="s">
         <v>319</v>
       </c>
@@ -9665,8 +10196,11 @@
         <f>HYPERLINK("1739962376_24_SPK_1_20250215_v2.1739611648.2264164.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C318" s="1" t="s">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" s="4" t="s">
         <v>320</v>
       </c>
@@ -9674,8 +10208,11 @@
         <f>HYPERLINK("1739962161_3_SPK_1_20250215_v2.1739603840.2258967.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C319" s="1" t="s">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" s="4" t="s">
         <v>321</v>
       </c>
@@ -9683,8 +10220,11 @@
         <f>HYPERLINK("1739962243_0_SPK_1_20250217_v2.1739806377.2388198.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C320" s="1" t="s">
+        <v>2032</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" s="4" t="s">
         <v>322</v>
       </c>
@@ -9692,8 +10232,11 @@
         <f>HYPERLINK("1739962494_10_SPK_1_20250217_v2.1739780189.2355491.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C321" s="1" t="s">
+        <v>2033</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" s="4" t="s">
         <v>323</v>
       </c>
@@ -9701,8 +10244,11 @@
         <f>HYPERLINK("1739961668_2_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C322" s="1" t="s">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323" s="4" t="s">
         <v>324</v>
       </c>
@@ -9710,8 +10256,11 @@
         <f>HYPERLINK("1739962998_16_SPK_0_20250216_v2.1739697766.2309766.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C323" s="1" t="s">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A324" s="4" t="s">
         <v>325</v>
       </c>
@@ -9719,8 +10268,11 @@
         <f>HYPERLINK("1739962175_3_SPK_1_20250215_v2.1739614093.2265728.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C324" s="1" t="s">
+        <v>2036</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" s="4" t="s">
         <v>326</v>
       </c>
@@ -9728,8 +10280,11 @@
         <f>HYPERLINK("1739962305_7_SPK_1_20250216_v2.1739695176.2307286.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C325" s="1" t="s">
+        <v>2037</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A326" s="4" t="s">
         <v>327</v>
       </c>
@@ -9737,8 +10292,11 @@
         <f>HYPERLINK("1739962962_0_SPK_1_20250217_v2.1739800434.2381527.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C326" s="1" t="s">
+        <v>2038</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327" s="4" t="s">
         <v>328</v>
       </c>
@@ -9746,8 +10304,11 @@
         <f>HYPERLINK("1739962416_0_SPK_1_20250216_v2.1739698726.2310851.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C327" s="1" t="s">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A328" s="4" t="s">
         <v>329</v>
       </c>
@@ -9755,8 +10316,11 @@
         <f>HYPERLINK("1739962432_2_SPK_0_20250215_v2.1739642412.2288835.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C328" s="1" t="s">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A329" s="4" t="s">
         <v>330</v>
       </c>
@@ -9764,8 +10328,11 @@
         <f>HYPERLINK("1739962447_4_SPK_1_20250216_v2.1739686917.2297991.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C329" s="1" t="s">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330" s="4" t="s">
         <v>331</v>
       </c>
@@ -9773,8 +10340,11 @@
         <f>HYPERLINK("1739962617_3_SPK_0_20250213_v2.1739461712.2231657.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C330" s="1" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331" s="4" t="s">
         <v>332</v>
       </c>
@@ -9782,8 +10352,11 @@
         <f>HYPERLINK("1739962239_7_SPK_0_20250216_v2.1739698265.2310367.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C331" s="1" t="s">
+        <v>2043</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332" s="4" t="s">
         <v>333</v>
       </c>
@@ -9791,8 +10364,11 @@
         <f>HYPERLINK("1739961624_4_SPK_1_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C332" s="1" t="s">
+        <v>2044</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333" s="4" t="s">
         <v>334</v>
       </c>
@@ -9800,8 +10376,11 @@
         <f>HYPERLINK("1739962256_7_SPK_0_20250217_v2.1739783441.2360167.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C333" s="1" t="s">
+        <v>2045</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334" s="4" t="s">
         <v>335</v>
       </c>
@@ -9810,7 +10389,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335" s="4" t="s">
         <v>336</v>
       </c>
@@ -9818,8 +10397,11 @@
         <f>HYPERLINK("1739962906_4_SPK_1_20250216_v2.1739710661.2333661.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="336" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C335" s="1" t="s">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A336" s="4" t="s">
         <v>337</v>
       </c>
@@ -9827,8 +10409,11 @@
         <f>HYPERLINK("1739962555_4_SPK_0_20250215_v2.1739634499.2284769.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="337" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C336" s="1" t="s">
+        <v>2046</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A337" s="4" t="s">
         <v>338</v>
       </c>
@@ -9837,7 +10422,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="338" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A338" s="4" t="s">
         <v>339</v>
       </c>
@@ -9845,8 +10430,11 @@
         <f>HYPERLINK("1739962266_14_SPK_0_20250215_v2.1739600840.2256930.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="339" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C338" s="1" t="s">
+        <v>2047</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339" s="4" t="s">
         <v>340</v>
       </c>
@@ -9854,8 +10442,11 @@
         <f>HYPERLINK("1739962654_6_SPK_0_20250215_v2.1739599940.2256629.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="340" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C339" s="1" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340" s="4" t="s">
         <v>341</v>
       </c>
@@ -9863,17 +10454,23 @@
         <f>HYPERLINK("1739962835_1_SPK_1_20250215_v2.1739625525.2280442.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="341" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C340" s="1" t="s">
+        <v>2049</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="B341" s="6" t="str">
+      <c r="B341" s="7" t="str">
         <f>HYPERLINK("1739961645_5_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="342" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C341" s="1" t="s">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342" s="4" t="s">
         <v>343</v>
       </c>
@@ -9881,8 +10478,11 @@
         <f>HYPERLINK("1739962409_1_SPK_1_20250218_v2.1739864349.2431631.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="343" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C342" s="1" t="s">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343" s="4" t="s">
         <v>344</v>
       </c>
@@ -9890,17 +10490,23 @@
         <f>HYPERLINK("1739962600_0_SPK_1_20250217_v2.1739810924.2392726.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="344" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C343" s="1" t="s">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A344" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="B344" s="6" t="str">
-        <f>HYPERLINK("1739962220_4_SPK_1_20250215_v2.1739616288.2269753.wav", "Play Audio")</f>
-        <v>Play Audio</v>
-      </c>
-    </row>
-    <row r="345" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B344" s="7" t="str">
+        <f>HYPERLINK("1739962220_4_SPK_1_20250215_v2.1739616288.2269753.C347wav", "Play Audio")</f>
+        <v>Play Audio</v>
+      </c>
+      <c r="C344" s="1" t="s">
+        <v>2054</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A345" s="4" t="s">
         <v>346</v>
       </c>
@@ -9908,8 +10514,11 @@
         <f>HYPERLINK("1739962614_3_SPK_0_20250215_v2.1739624456.2279776.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="346" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C345" s="1" t="s">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346" s="4" t="s">
         <v>347</v>
       </c>
@@ -9917,8 +10526,11 @@
         <f>HYPERLINK("1739962753_7_SPK_1_20250217_v2.1739783930.2360950.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="347" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C346" s="1" t="s">
+        <v>2056</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A347" s="4" t="s">
         <v>348</v>
       </c>
@@ -9926,8 +10538,11 @@
         <f>HYPERLINK("1739962826_9_SPK_1_20250215_v2.1739596848.2256007.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="348" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C347" s="1" t="s">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A348" s="4" t="s">
         <v>349</v>
       </c>
@@ -9935,8 +10550,11 @@
         <f>HYPERLINK("1739962906_1_SPK_0_20250216_v2.1739710661.2333661.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="349" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C348" s="1" t="s">
+        <v>2058</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A349" s="4" t="s">
         <v>350</v>
       </c>
@@ -9944,8 +10562,11 @@
         <f>HYPERLINK("1739962399_10_SPK_1_20250213_v2.1739454160.2223094.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="350" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C349" s="1" t="s">
+        <v>2059</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A350" s="4" t="s">
         <v>351</v>
       </c>
@@ -9953,8 +10574,11 @@
         <f>HYPERLINK("1739962791_3_SPK_1_20250215_v2.1739610541.2263379.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="351" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C350" s="1" t="s">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A351" s="4" t="s">
         <v>352</v>
       </c>
@@ -9962,8 +10586,11 @@
         <f>HYPERLINK("1739962614_2_SPK_0_20250215_v2.1739624456.2279776.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="352" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C351" s="1" t="s">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A352" s="4" t="s">
         <v>353</v>
       </c>
@@ -9971,8 +10598,11 @@
         <f>HYPERLINK("1739962216_4_SPK_0_20250215_v2.1739616465.2270610.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="353" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C352" s="1" t="s">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A353" s="4" t="s">
         <v>354</v>
       </c>
@@ -9980,8 +10610,11 @@
         <f>HYPERLINK("1739962933_4_SPK_1_20250215_v2.1739604548.2259402.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="354" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C353" s="1" t="s">
+        <v>2063</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A354" s="4" t="s">
         <v>355</v>
       </c>
@@ -9989,8 +10622,11 @@
         <f>HYPERLINK("1739962266_17_SPK_1_20250215_v2.1739600840.2256930.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="355" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C354" s="1" t="s">
+        <v>2064</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A355" s="4" t="s">
         <v>356</v>
       </c>
@@ -9998,8 +10634,11 @@
         <f>HYPERLINK("1739962955_8_SPK_1_20250213_v2.1739439090.2205291.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="356" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C355" s="1" t="s">
+        <v>2065</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A356" s="4" t="s">
         <v>357</v>
       </c>
@@ -10007,8 +10646,11 @@
         <f>HYPERLINK("1739962144_14_SPK_1_20250215_v2.1739639895.2287671.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="357" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C356" s="1" t="s">
+        <v>2066</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A357" s="4" t="s">
         <v>358</v>
       </c>
@@ -10016,8 +10658,11 @@
         <f>HYPERLINK("1739962736_4_SPK_0_20250213_v2.1739446911.2214794.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="358" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C357" s="1" t="s">
+        <v>1854</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A358" s="4" t="s">
         <v>359</v>
       </c>
@@ -10025,8 +10670,11 @@
         <f>HYPERLINK("1739962759_7_SPK_1_20250218_v2.1739862982.2429599.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="359" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C358" s="1" t="s">
+        <v>2067</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A359" s="4" t="s">
         <v>360</v>
       </c>
@@ -10034,8 +10682,11 @@
         <f>HYPERLINK("1739962940_2_SPK_0_20250213_v2.1739444021.2211593.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="360" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C359" s="1" t="s">
+        <v>2068</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A360" s="4" t="s">
         <v>361</v>
       </c>
@@ -10043,8 +10694,11 @@
         <f>HYPERLINK("1739962416_11_SPK_1_20250216_v2.1739698726.2310851.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="361" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C360" s="1" t="s">
+        <v>2069</v>
+      </c>
+    </row>
+    <row r="361" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A361" s="4" t="s">
         <v>362</v>
       </c>
@@ -10052,8 +10706,11 @@
         <f>HYPERLINK("1739962358_1_SPK_0_20250216_v2.1739715775.2337113.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="362" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C361" s="1" t="s">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A362" s="4" t="s">
         <v>363</v>
       </c>
@@ -10061,8 +10718,11 @@
         <f>HYPERLINK("1739962555_1_SPK_0_20250215_v2.1739634499.2284769.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="363" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C362" s="1" t="s">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A363" s="4" t="s">
         <v>364</v>
       </c>
@@ -10070,8 +10730,11 @@
         <f>HYPERLINK("1739962354_2_SPK_1_20250216_v2.1739698639.2310716.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="364" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C363" s="1" t="s">
+        <v>2072</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A364" s="4" t="s">
         <v>365</v>
       </c>
@@ -10079,8 +10742,11 @@
         <f>HYPERLINK("1739962555_0_SPK_0_20250215_v2.1739634499.2284769.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="365" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C364" s="1" t="s">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A365" s="4" t="s">
         <v>366</v>
       </c>
@@ -10088,8 +10754,11 @@
         <f>HYPERLINK("1739962532_3_SPK_1_20250217_v2.1739782872.2359341.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="366" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C365" s="1" t="s">
+        <v>2074</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A366" s="4" t="s">
         <v>367</v>
       </c>
@@ -10097,8 +10766,11 @@
         <f>HYPERLINK("1739962709_0_SPK_0_20250217_v2.1739780534.2356086.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="367" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C366" s="1" t="s">
+        <v>2075</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A367" s="4" t="s">
         <v>368</v>
       </c>
@@ -10106,8 +10778,11 @@
         <f>HYPERLINK("1739962622_1_SPK_0_20250216_v2.1739720481.2339514.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="368" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C367" s="1" t="s">
+        <v>2076</v>
+      </c>
+    </row>
+    <row r="368" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A368" s="4" t="s">
         <v>369</v>
       </c>
@@ -10115,8 +10790,11 @@
         <f>HYPERLINK("1739962861_1_SPK_0_20250216_v2.1739695895.2308017.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="369" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C368" s="1" t="s">
+        <v>2077</v>
+      </c>
+    </row>
+    <row r="369" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A369" s="4" t="s">
         <v>370</v>
       </c>
@@ -10124,8 +10802,11 @@
         <f>HYPERLINK("1739962699_3_SPK_0_20250216_v2.1739705425.2330497.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="370" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C369" s="1" t="s">
+        <v>2078</v>
+      </c>
+    </row>
+    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A370" s="4" t="s">
         <v>371</v>
       </c>
@@ -10133,8 +10814,11 @@
         <f>HYPERLINK("1739962275_3_SPK_0_20250217_v2.1739779643.2354689.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="371" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C370" s="1" t="s">
+        <v>2079</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A371" s="4" t="s">
         <v>372</v>
       </c>
@@ -10142,8 +10826,11 @@
         <f>HYPERLINK("1739962586_6_SPK_1_20250215_v2.1739597847.2256179.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="372" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C371" s="1" t="s">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A372" s="4" t="s">
         <v>373</v>
       </c>
@@ -10151,8 +10838,11 @@
         <f>HYPERLINK("1739962561_0_SPK_0_20250217_v2.1739786281.2364487.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="373" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C372" s="1" t="s">
+        <v>2081</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A373" s="4" t="s">
         <v>374</v>
       </c>
@@ -10160,8 +10850,11 @@
         <f>HYPERLINK("1739962405_6_SPK_0_20250215_v2.1739608747.2261893.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="374" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C373" s="1" t="s">
+        <v>2082</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A374" s="4" t="s">
         <v>375</v>
       </c>
@@ -10169,8 +10862,11 @@
         <f>HYPERLINK("1739962459_21_SPK_1_20250216_v2.1739696150.2308305.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="375" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C374" s="1" t="s">
+        <v>2083</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A375" s="4" t="s">
         <v>376</v>
       </c>
@@ -10178,8 +10874,11 @@
         <f>HYPERLINK("1739962642_9_SPK_1_20250218_v2.1739864664.2432073.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="376" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C375" s="1" t="s">
+        <v>2084</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A376" s="4" t="s">
         <v>377</v>
       </c>
@@ -10187,8 +10886,11 @@
         <f>HYPERLINK("1739962576_2_SPK_0_20250216_v2.1739695278.2307344.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="377" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C376" s="1" t="s">
+        <v>2085</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A377" s="4" t="s">
         <v>378</v>
       </c>
@@ -10196,8 +10898,11 @@
         <f>HYPERLINK("1739962447_0_SPK_0_20250216_v2.1739686917.2297991.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="378" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C377" s="1" t="s">
+        <v>2086</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A378" s="4" t="s">
         <v>379</v>
       </c>
@@ -10205,8 +10910,11 @@
         <f>HYPERLINK("1739962405_0_SPK_1_20250215_v2.1739608747.2261893.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="379" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C378" s="1" t="s">
+        <v>2087</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A379" s="4" t="s">
         <v>380</v>
       </c>
@@ -10214,8 +10922,11 @@
         <f>HYPERLINK("1739962459_20_SPK_1_20250216_v2.1739696150.2308305.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="380" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C379" s="1" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A380" s="4" t="s">
         <v>381</v>
       </c>
@@ -10223,8 +10934,11 @@
         <f>HYPERLINK("1739962981_8_SPK_0_20250215_v2.1739611404.2264001.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="381" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C380" s="1" t="s">
+        <v>2089</v>
+      </c>
+    </row>
+    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A381" s="4" t="s">
         <v>382</v>
       </c>
@@ -10232,8 +10946,11 @@
         <f>HYPERLINK("1739962220_7_SPK_0_20250215_v2.1739616288.2269753.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="382" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C381" s="1" t="s">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A382" s="4" t="s">
         <v>383</v>
       </c>
@@ -10241,8 +10958,11 @@
         <f>HYPERLINK("1739962447_12_SPK_1_20250216_v2.1739686917.2297991.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="383" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C382" s="1" t="s">
+        <v>2091</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A383" s="4" t="s">
         <v>384</v>
       </c>
@@ -10250,8 +10970,11 @@
         <f>HYPERLINK("1739962148_5_SPK_0_20250215_v2.1739601562.2257186.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="384" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C383" s="1" t="s">
+        <v>2092</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A384" s="4" t="s">
         <v>385</v>
       </c>
@@ -10259,8 +10982,11 @@
         <f>HYPERLINK("1739962693_3_SPK_1_20250218_v2.1739864856.2432292.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="385" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C384" s="1" t="s">
+        <v>2093</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A385" s="4" t="s">
         <v>386</v>
       </c>
@@ -10268,8 +10994,11 @@
         <f>HYPERLINK("1739961641_20_SPK_0_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="386" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C385" s="1" t="s">
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A386" s="4" t="s">
         <v>387</v>
       </c>
@@ -10277,8 +11006,11 @@
         <f>HYPERLINK("1739962232_0_SPK_1_20250215_v2.1739627725.2281684.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="387" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C386" s="1" t="s">
+        <v>2095</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A387" s="4" t="s">
         <v>388</v>
       </c>
@@ -10286,8 +11018,11 @@
         <f>HYPERLINK("1739962479_0_SPK_1_20250215_v2.1739610716.2263497.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="388" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C387" s="1" t="s">
+        <v>2096</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A388" s="4" t="s">
         <v>389</v>
       </c>
@@ -10296,7 +11031,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="389" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A389" s="4" t="s">
         <v>390</v>
       </c>
@@ -10304,8 +11039,11 @@
         <f>HYPERLINK("1739962432_15_SPK_0_20250215_v2.1739642412.2288835.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="390" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C389" s="1" t="s">
+        <v>2097</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A390" s="4" t="s">
         <v>391</v>
       </c>
@@ -10313,8 +11051,11 @@
         <f>HYPERLINK("1739962742_0_SPK_0_20250217_v2.1739786644.2364947.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="391" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C390" s="1" t="s">
+        <v>2098</v>
+      </c>
+    </row>
+    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A391" s="4" t="s">
         <v>392</v>
       </c>
@@ -10323,7 +11064,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="392" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392" s="4" t="s">
         <v>393</v>
       </c>
@@ -10331,8 +11072,11 @@
         <f>HYPERLINK("1739961698_0_SPK_1_20250213_v2.1739437852.2203015.wav", "Play Audio")</f>
         <v>Play Audio</v>
       </c>
-    </row>
-    <row r="393" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C392" s="1" t="s">
+        <v>2099</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A393" s="4" t="s">
         <v>394</v>
       </c>
@@ -10341,7 +11085,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="394" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A394" s="4" t="s">
         <v>395</v>
       </c>
@@ -10350,7 +11094,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="395" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A395" s="4" t="s">
         <v>396</v>
       </c>
@@ -10359,7 +11103,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="396" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A396" s="4" t="s">
         <v>397</v>
       </c>
@@ -10368,7 +11112,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="397" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A397" s="4" t="s">
         <v>398</v>
       </c>
@@ -10377,7 +11121,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="398" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A398" s="4" t="s">
         <v>399</v>
       </c>
@@ -10386,7 +11130,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="399" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A399" s="4" t="s">
         <v>400</v>
       </c>
@@ -10395,7 +11139,7 @@
         <v>Play Audio</v>
       </c>
     </row>
-    <row r="400" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A400" s="4" t="s">
         <v>401</v>
       </c>

</xml_diff>